<commit_message>
referenceRange limited to ..1 5191ae2febf61530131c93f964a55ad99de82d3d
</commit_message>
<xml_diff>
--- a/nr-add-lipids/ig/StructureDefinition-mesures-observation-cholesterol-aspect.xlsx
+++ b/nr-add-lipids/ig/StructureDefinition-mesures-observation-cholesterol-aspect.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-01-20T10:06:11+00:00</t>
+    <t>2026-01-20T11:11:06+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -8426,7 +8426,7 @@
         <v>80</v>
       </c>
       <c r="G53" t="s" s="2">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="H53" t="s" s="2">
         <v>94</v>

</xml_diff>